<commit_message>
06.05. First Web Regression
</commit_message>
<xml_diff>
--- a/testdata/configuration.xlsx
+++ b/testdata/configuration.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="10187"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -143,7 +143,7 @@
     <t>dev</t>
   </si>
   <si>
-    <t>https://uat.dbp.nlbkb.rs/login</t>
+    <t>https://test.dbp.nlbkb.rs/login</t>
   </si>
   <si>
     <t>Chrome</t>
@@ -161,10 +161,10 @@
     <t>1</t>
   </si>
   <si>
-    <t>rs.nlb.klik.uat:id/</t>
-  </si>
-  <si>
-    <t>rs.nlb.klik.uat</t>
+    <t>si.nlb.klik.uat:id/</t>
+  </si>
+  <si>
+    <t>si.nlb.klik.uat</t>
   </si>
   <si>
     <t>si.nlb.klik.RootActivity</t>
@@ -1331,7 +1331,6 @@
     <col min="8" max="9" width="22.5740740740741" customWidth="1"/>
     <col min="10" max="12" width="31.712962962963" customWidth="1"/>
     <col min="13" max="13" width="16.4259259259259" customWidth="1"/>
-    <col min="14" max="14" width="22.5555555555556" customWidth="1"/>
     <col min="20" max="20" width="16.4259259259259" customWidth="1"/>
     <col min="21" max="21" width="12.287037037037" customWidth="1"/>
     <col min="31" max="31" width="16" customWidth="1"/>
@@ -1567,7 +1566,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="AF2" r:id="rId1" display="bozidar.tomasevic@dtc.rs"/>
-    <hyperlink ref="C2" r:id="rId2" display="https://uat.dbp.nlbkb.rs/login" tooltip="https://uat.dbp.nlbkb.rs/login"/>
+    <hyperlink ref="C2" r:id="rId2" display="https://test.dbp.nlbkb.rs/login" tooltip="https://test.dbp.nlbkb.rs/login"/>
     <hyperlink ref="AI2" r:id="rId3" display="\\10.11.1.158\03. TEST Team\NLB SLO\FileShare\UAT" tooltip="\\10.11.1.158\03. TEST Team\NLB SLO\FileShare\UAT"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
01.06. Sa drugog kompa
</commit_message>
<xml_diff>
--- a/testdata/configuration.xlsx
+++ b/testdata/configuration.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="10187"/>
+    <workbookView windowWidth="20490" windowHeight="7500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1321,20 +1321,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:AK2"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="9.22222222222222" customWidth="1"/>
+    <col min="1" max="1" width="9.21904761904762" customWidth="1"/>
     <col min="2" max="2" width="13.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="28.1111111111111" customWidth="1"/>
-    <col min="4" max="5" width="22.5555555555556" customWidth="1"/>
+    <col min="3" max="3" width="28.1142857142857" customWidth="1"/>
+    <col min="4" max="5" width="22.552380952381" customWidth="1"/>
     <col min="7" max="7" width="20.3333333333333" customWidth="1"/>
-    <col min="8" max="9" width="22.5740740740741" customWidth="1"/>
-    <col min="10" max="12" width="31.712962962963" customWidth="1"/>
-    <col min="13" max="13" width="16.4259259259259" customWidth="1"/>
-    <col min="20" max="20" width="16.4259259259259" customWidth="1"/>
-    <col min="21" max="21" width="12.287037037037" customWidth="1"/>
+    <col min="8" max="9" width="22.5714285714286" customWidth="1"/>
+    <col min="10" max="12" width="31.7142857142857" customWidth="1"/>
+    <col min="13" max="13" width="16.4285714285714" customWidth="1"/>
+    <col min="20" max="20" width="16.4285714285714" customWidth="1"/>
+    <col min="21" max="21" width="12.2857142857143" customWidth="1"/>
     <col min="31" max="31" width="16" customWidth="1"/>
-    <col min="32" max="32" width="17.712962962963" customWidth="1"/>
+    <col min="32" max="32" width="17.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37">

</xml_diff>